<commit_message>
Run with num_walks=60,  walk_length=15, p=3, q=1
</commit_message>
<xml_diff>
--- a/results/CA/deepwalk_embedding_size_results.xlsx
+++ b/results/CA/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8288058361033812</v>
+        <v>0.821119184319777</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8282583746954908</v>
+        <v>0.8252545443467152</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8311561581201998</v>
+        <v>0.8242428071148732</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8314903954067313</v>
+        <v>0.8244511558223995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run with --num-walks 50 --walk-length 15 --p 3 --q 1
</commit_message>
<xml_diff>
--- a/results/CA/deepwalk_embedding_size_results.xlsx
+++ b/results/CA/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.821119184319777</v>
+        <v>0.8207601758169121</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8252545443467152</v>
+        <v>0.8241124099079512</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8242428071148732</v>
+        <v>0.827026316819809</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8244511558223995</v>
+        <v>0.8248107142569168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
num-walks 50 --walk-length 15 --p 3 --q 1
CA: so so, MHD not bad
</commit_message>
<xml_diff>
--- a/results/CA/deepwalk_embedding_size_results.xlsx
+++ b/results/CA/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8207601758169121</v>
+        <v>0.8136169232075161</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8241124099079512</v>
+        <v>0.8101025562657439</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.827026316819809</v>
+        <v>0.8025647216170437</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8248107142569168</v>
+        <v>0.791501854337034</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Using only geo features
</commit_message>
<xml_diff>
--- a/results/CA/deepwalk_embedding_size_results.xlsx
+++ b/results/CA/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8136169232075161</v>
+        <v>0.8173510335850909</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8101025562657439</v>
+        <v>0.8200135237358518</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8025647216170437</v>
+        <v>0.8210501297135518</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.791501854337034</v>
+        <v>0.8231692386433485</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
num-walks 5 --walk-length 10 --p 2 --q 2
grid search on p,q
</commit_message>
<xml_diff>
--- a/results/CA/deepwalk_embedding_size_results.xlsx
+++ b/results/CA/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8173510335850909</v>
+        <v>0.8175192578027209</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8200135237358518</v>
+        <v>0.8197175808016233</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8210501297135518</v>
+        <v>0.8230822040446923</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8231692386433485</v>
+        <v>0.8207877941150606</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore project to state at commit 8ba9af0 - paper draft
</commit_message>
<xml_diff>
--- a/results/CA/deepwalk_embedding_size_results.xlsx
+++ b/results/CA/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8175192578027209</v>
+        <v>0.8288058361033812</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8197175808016233</v>
+        <v>0.8282583746954908</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8230822040446923</v>
+        <v>0.8311561581201998</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8207877941150606</v>
+        <v>0.8314903954067313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Re-run on 3090 - bad for MHD !
</commit_message>
<xml_diff>
--- a/results/CA/deepwalk_embedding_size_results.xlsx
+++ b/results/CA/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8288058361033812</v>
+        <v>0.828281354052949</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8282583746954908</v>
+        <v>0.8261044227814246</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8311561581201998</v>
+        <v>0.8306026376045443</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8314903954067313</v>
+        <v>0.8356585173700486</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert to last kNN
</commit_message>
<xml_diff>
--- a/results/CA/deepwalk_embedding_size_results.xlsx
+++ b/results/CA/deepwalk_embedding_size_results.xlsx
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.828281354052949</v>
+        <v>0.8175192578027209</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8261044227814246</v>
+        <v>0.8197175808016233</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8306026376045443</v>
+        <v>0.8230822040446923</v>
       </c>
     </row>
     <row r="5">
@@ -469,7 +469,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8356585173700486</v>
+        <v>0.8207877941150606</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
num-walks 20 --walk-length 15 --p 2 --q 2
Run on the whole MHD dataset
</commit_message>
<xml_diff>
--- a/results/CA/deepwalk_embedding_size_results.xlsx
+++ b/results/CA/deepwalk_embedding_size_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8189752385217032</v>
+        <v>0.8191798470894323</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8218938782466065</v>
+        <v>0.8228423045296026</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,15 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8248316939317709</v>
+        <v>0.8257144193141382</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.8265323258209694</v>
       </c>
     </row>
   </sheetData>

</xml_diff>